<commit_message>
Update prepare-documents NT prerequisites from BPMN
Align ump-prepare-documents-ncins-pa NT workbook with actual BPMN job
types, call activity mapping, and STATIC/DYNAMIC inputs from PR BPMN.

Co-authored-by: Дмитрий Григорьев <pulya-na-vullet@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/nt-prerequisites-xlsx/НТ пререквизиты __ Worker ump-prepare-documents-ncins-pa.xlsx
+++ b/nt-prerequisites-xlsx/НТ пререквизиты __ Worker ump-prepare-documents-ncins-pa.xlsx
@@ -11,6 +11,7 @@
     <sheet name="1. Согласование" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="2. Минимальная информация" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="3. Полная информация" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="BPMN методы (источник)" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -464,7 +465,7 @@
   <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="100" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -477,7 +478,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>UMP · 21 июля 2026</t>
+          <t>UMP · 21 июля 2026 · актуализировано по BPMN ump-prepare-documents-ncins-pa</t>
         </is>
       </c>
     </row>
@@ -512,7 +513,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Назначение: Формирования документов</t>
+          <t>Назначение: Процесс подготовки документов (ncins). Источник правды по шагам: BPMN ump-prepare-documents-ncins-pa.bpmn (PR NCINS-143).</t>
         </is>
       </c>
     </row>
@@ -548,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>UMP · 21 июля 2026</t>
+          <t>UMP · 21 июля 2026 · актуализировано по BPMN ump-prepare-documents-ncins-pa</t>
         </is>
       </c>
     </row>
@@ -620,7 +621,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>UMP · 21 июля 2026</t>
+          <t>UMP · 21 июля 2026 · актуализировано по BPMN ump-prepare-documents-ncins-pa</t>
         </is>
       </c>
     </row>
@@ -663,7 +664,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="108" customHeight="1">
+    <row r="6" ht="160" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
         <is>
           <t>1</t>
@@ -676,12 +677,19 @@
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>[ump-prepare-documents-ncins-pa] Формирования документов: Start → Service Task get-application-data (GET /applications/{id}) → Service Task подготовка reportData для ПФ → Call Activity generate/save AlfaCapture (POST /documents/generate) → Service Task update-product (PUT /products/{id}, contractLink) → End.</t>
+          <t>[ump-prepare-documents-ncins-pa] Процесс подготовки документов (BPMN).
+Цепочка шагов (из BPMN):
+1) StartEvent
+2) Service Task service-task-get-params «Получить данные по заявке» — zeebe type get-application-data; input processType=PREPARE_DOCUMENTS (STATIC)
+3) Service Task service-task-get-report-data «Подготовить данные для ПФ» — type ump-prepare-documents-ncins-pa.get-report-data
+4) Call Activity call-activity-ump-generate-and-save-document-pa «Формирование и сохранение документа в AlfaCapture» — called process ump-generate-and-save-document-pa
+5) Service Task service-task-update-product «Обновить данные по продукту» — type update-product
+6) EndEvent</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>Confluence/BPMN ump-prepare-documents-ncins-pa</t>
+          <t>Файл: bpmn/src/main/resources/ump-ncins-pa/ump-prepare-documents-ncins-pa.bpmn</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
@@ -708,7 +716,7 @@
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>Процесс синхронный. СА: единый SLA на sync-методы — несколько секунд на каждый вызов. Точное число — TBD с НТ.</t>
+          <t>Все шаги синхронные (service task / call activity). По ответам СА: единый SLA на sync — несколько секунд на вызов. Точное число — TBD с НТ.</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
@@ -727,7 +735,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="54" customHeight="1">
+    <row r="8" ht="72" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
           <t>3</t>
@@ -740,12 +748,12 @@
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>От общей базы 15000 заявок/мес. Среднее ≈ 89/час; макс (пик) ≈ 180/час. На заявку генерится 1 файл. Пример размера reportData/файла ≈ 283 КБ (avg/p95/max — TBD).</t>
+          <t>От общей базы 15000 заявок/мес (SFA, рабочие часы). Среднее ≈ 89/час; максимальное (пик ×2) ≈ 180/час. 1 документ на заявку. Пример размера файла/reportData ≈ 283 КБ (avg/p95/max — TBD).</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>15000/мес, рабочие часы; 1 документ на заявку</t>
+          <t>Способ: 15000/~21 р.д./8 ч ≈ 89/час; пик экспертно ×2</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
@@ -759,7 +767,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="45" customHeight="1">
+    <row r="9" ht="50" customHeight="1">
       <c r="A9" s="8" t="inlineStr">
         <is>
           <t>4</t>
@@ -772,12 +780,12 @@
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>TBD (прогноз через 6 мес не зафиксирован командой)</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>TBD макс/среднее через 6 мес</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
@@ -791,7 +799,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="90" customHeight="1">
+    <row r="10" ht="126" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
         <is>
           <t>5</t>
@@ -804,16 +812,17 @@
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>[GET /applications/{id}] ump-application-facade ~89–180/час
-[Подготовка данных для ПФ / reportData] ~89–180/час
-[POST /documents/generate] OBIP+AlfaCapture ~89–180/час
-[PUT /products/{id}] ump-products ~89–180/час
+          <t>Сервис/метод | ЧПН (ср./пик, вызовов/час) — оценка от ЧПН процесса:
+[get-application-data] GET заявка ~89 / ~180
+[ump-prepare-documents-ncins-pa.get-report-data] подготовка ПФ ~89 / ~180
+[ump-generate-and-save-document-pa] Call Activity (генерация+AC) ~89 / ~180
+[update-product] обновление продукта ~89 / ~180
 Лимит параллелизма: 200 потоков (бэкенд)</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>Может совпадать с ЧПН процесса</t>
+          <t>Может совпадать с ЧПН процесса (каждый шаг 1 раз на заявку)</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
@@ -827,7 +836,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="45" customHeight="1">
+    <row r="11" ht="50" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
           <t>6</t>
@@ -840,7 +849,7 @@
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>TBD (пропорционально п.4)</t>
+          <t>TBD (пропорционально п.4). Пока ориентир = п.5.</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
@@ -896,7 +905,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>UMP · 21 июля 2026</t>
+          <t>UMP · 21 июля 2026 · актуализировано по BPMN ump-prepare-documents-ncins-pa</t>
         </is>
       </c>
     </row>
@@ -939,7 +948,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="126" customHeight="1">
+    <row r="6" ht="160" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
         <is>
           <t>6</t>
@@ -952,15 +961,23 @@
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>У воркера нет отдельного HTTP API процесса. Старт из main Call Activity / Camunda:
-variables: businessKey (DYNAMIC), productCode=NON_CREDIT_INSURANCE (const для продукта).
-Внутри: GET /applications/{id}?include=PARTICIPANT,PRODUCT — id=businessKey; include=STATIC.
-PUT /products/{id} — id=productId из заявки; в теле фактически значимо contractLink из AC.</t>
+          <t>У процесса нет HTTP-эндпоинта. Запуск через Camunda/Zeebe (из main Call Activity или напрямую).
+Входные переменные процесса на старте:
+- businessKey — DYNAMIC (UUID заявки)
+- productCode — передаётся на старте; для ncins фактически STATIC = NON_CREDIT_INSURANCE
+Маппинг Call Activity ump-generate-and-save-document-pa (из BPMN):
+- serviceId = businessKey (DYNAMIC)
+- serviceCode = "APPLICATION" (STATIC)
+- productCode = productCode (DYNAMIC_START / фактически const продукта)
+- documents = documents (DYNAMIC, из get-report-data)
+Outputs: docsResult←result, acRequestId, acDocuments
+get-application-data: input processType = PREPARE_DOCUMENTS (STATIC)
+update-product: type update-product (после AC)</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>Параметризация businessKey/заявок на объём ≥ ЧПН; productCode const.</t>
+          <t>Параметризация: набор businessKey ≥ ЧПН; productCode/serviceCode/processType — константы</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
@@ -974,7 +991,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="54" customHeight="1">
+    <row r="7" ht="108" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
         <is>
           <t>7</t>
@@ -987,14 +1004,15 @@
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>Успех процесса: result=SUCCESS.
-get-application: getProcessParams=SUCCESS|ERROR.
-Ошибки генерации ПФ (бэкенд): HTTP 400 и 500 (полный каталог тел — у Жени/НИБ TBD).</t>
+          <t>Ожидаемый успешный ход: все task SUCCESS, процесс доходит до End.
+Call Activity возвращает: docsResult, acRequestId, acDocuments.
+Ошибки генерации ПФ/AC (из ответов бэкенда): HTTP 400 и 500 (полный каталог тел — TBD у Жени).
+get-application-data: getProcessParams=SUCCESS|ERROR (по процессной доке).</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>200/успех Camunda SUCCESS; 400/500 на generate</t>
+          <t>SUCCESS / ERROR; 400; 500</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
@@ -1008,7 +1026,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="54" customHeight="1">
+    <row r="8" ht="90" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
           <t>8</t>
@@ -1021,12 +1039,12 @@
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>PUT /products/{id}: формально full update; по смыслу добавляется/обновляется поле contractLink (подтверждено бэкендом). Side effects сверх этого не выделялись.</t>
+          <t>Шаг update-product (type update-product): обновляет продукт; по ответам СА/бэкенда фактически значимо поле contractLink (формально PUT обновляет запись). Данные заявки читаются в get-application-data, не пишутся обратно в UMP кроме update-product.</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>Обновляется contractLink у продукта</t>
+          <t>contractLink у продукта (+ поля product из маппинга update-product)</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
@@ -1040,7 +1058,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="45" customHeight="1">
+    <row r="9" ht="50" customHeight="1">
       <c r="A9" s="8" t="inlineStr">
         <is>
           <t>9</t>
@@ -1072,7 +1090,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="54" customHeight="1">
+    <row r="10" ht="90" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
         <is>
           <t>10</t>
@@ -1085,12 +1103,12 @@
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>ПФ/AlfaCapture — решение по мокам на стенде НТ уточнить (без AC своей папки реальное сохранение ограничено). Ошибки 400/500 иметь в негативных сценариях.</t>
+          <t>Внешние вызовы через Call Activity ump-generate-and-save-document-pa (ПФ + AlfaCapture). На НТ моки/доступ к AC уточнять: без своей папки AC реальное сохранение ограничено. get-application-data и update-product — внутренние job types UMP.</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>Мок/стенд ПФ+AC по договорённости с НТ</t>
+          <t>Мок/стенд для ump-generate-and-save-document-pa при необходимости</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
@@ -1104,7 +1122,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="45" customHeight="1">
+    <row r="11" ht="50" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
           <t>11</t>
@@ -1117,12 +1135,12 @@
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>Как у sync: несколько секунд на вызов (TBD точное значение с НТ).</t>
+          <t>Как у sync: несколько секунд на вызов (TBD точное значение с НТ), включая call activity generate/save.</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>generate/save ~несколько сек</t>
+          <t>get-report-data / generate-and-save / update-product — по несколько сек</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
@@ -1136,7 +1154,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="72" customHeight="1">
+    <row r="12" ht="126" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
         <is>
           <t>12</t>
@@ -1149,16 +1167,19 @@
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>1) Success: get→prepare reportData→generate+save→PUT product→SUCCESS.
-2) GET 4xx → getProcessParams=ERROR.
-3) GET 5xx → 3 ретрая ×1с → инцидент.
-4) Generate 400/500.
-5) Пик в лимите 200 потоков.</t>
+          <t>Строго по BPMN (последовательность):
+1) Start
+2) get-application-data (processType=PREPARE_DOCUMENTS)
+3) ump-prepare-documents-ncins-pa.get-report-data
+4) Call Activity ump-generate-and-save-document-pa (serviceCode=APPLICATION)
+5) update-product
+6) End
+Негатив: ошибка get-application-data; ошибка generate 400/500; пик в лимите 200 потоков.</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>Последовательные sync-вызовы внутри одного процесса на заявку</t>
+          <t>Один бизнес-процесс = последовательный вызов 4 исполняемых шагов</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
@@ -1169,6 +1190,278 @@
       <c r="F12" s="8" t="inlineStr">
         <is>
           <t>Аналитик</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A4:F4"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>НТ пререквизиты :: Worker ump-prepare-documents-ncins-pa</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>UMP · 21 июля 2026 · актуализировано по BPMN ump-prepare-documents-ncins-pa</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Шаги из ump-prepare-documents-ncins-pa.bpmn — STATIC vs DYNAMIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>BPMN id</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Type / called process</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>Ключевые параметры</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>STATIC / DYNAMIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="55" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>StartEvent_1</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Start</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>startEvent</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>ожидает vars процесса</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>DYNAMIC_START: businessKey, productCode</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="55" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>service-task-get-params</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Получить данные по заявке</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>zeebe type: get-application-data</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>processType → PREPARE_DOCUMENTS</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>STATIC: processType=PREPARE_DOCUMENTS; DYNAMIC_START: businessKey (для GET)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="55" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>service-task-get-report-data</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>Подготовить данные для ПФ</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>type: ump-prepare-documents-ncins-pa.get-report-data</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>формирует documents/reportData</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>DYNAMIC_FROM_APP/PREV → documents</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="55" customHeight="1">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>call-activity-ump-generate-and-save-document-pa</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Формирование и сохранение документа в AlfaCapture</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>calledElement: ump-generate-and-save-document-pa</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>serviceId=businessKey; serviceCode="APPLICATION"; productCode; documents; out: docsResult, acRequestId, acDocuments</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>STATIC: serviceCode=APPLICATION; DYNAMIC: serviceId, productCode, documents</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="55" customHeight="1">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>service-task-update-product</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Обновить данные по продукту</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>type: update-product</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>после AC</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>DYNAMIC_FROM_PREV: acDocuments/links → product update</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="55" customHeight="1">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Event_16wgp78</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>End</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>endEvent</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>

</xml_diff>